<commit_message>
updated system core requirements
</commit_message>
<xml_diff>
--- a/docs/NAO_requirements.xlsx
+++ b/docs/NAO_requirements.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\admin\Desktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2653510A-8AD2-4C8C-A046-315B1A913FC6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3C8674D0-B0EF-4203-A2F5-9DD01D6D145E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="6700" yWindow="2790" windowWidth="29430" windowHeight="15380" firstSheet="5" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="7040" yWindow="3130" windowWidth="29430" windowHeight="15380" firstSheet="5" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="User Access &amp; Login" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="304" uniqueCount="171">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="299" uniqueCount="169">
   <si>
     <t>ID</t>
   </si>
@@ -130,45 +130,30 @@
     <t>SR-VOICE-01</t>
   </si>
   <si>
-    <t>NAO shall be the primary student voice-input device when the robot is technically operational.</t>
-  </si>
-  <si>
     <t>Client explicitly prefers NAO as the primary interaction device.</t>
   </si>
   <si>
     <t>SR-VOICE-02</t>
   </si>
   <si>
-    <t>NAO shall capture a student's spoken enquiry as an audio recording suitable for transmission to the backend.</t>
-  </si>
-  <si>
     <t>Required by agreed audio-file architecture.</t>
   </si>
   <si>
     <t>SR-VOICE-03</t>
   </si>
   <si>
-    <t>The client device shall transmit the captured audio file to the Mac Studio backend using HTTP.</t>
-  </si>
-  <si>
     <t>Client/team architecture decision.</t>
   </si>
   <si>
     <t>SR-VOICE-04</t>
   </si>
   <si>
-    <t>Each submitted audio request shall receive a success or failure response from the backend.</t>
-  </si>
-  <si>
     <t>Required to detect network/upload failures.</t>
   </si>
   <si>
     <t>SR-VOICE-05</t>
   </si>
   <si>
-    <t>If NAO cannot be made operational, the system shall support an iPad fallback that can record student audio, upload the recording to the Mac Studio and display the returned text response.</t>
-  </si>
-  <si>
     <t>Client-approved fallback approach.</t>
   </si>
   <si>
@@ -198,9 +183,6 @@
     <t>SR-STT-01</t>
   </si>
   <si>
-    <t>The Mac Studio backend shall convert a received audio recording into text before submitting the enquiry to the LLM.</t>
-  </si>
-  <si>
     <t>Agreed backend architecture.</t>
   </si>
   <si>
@@ -269,18 +251,12 @@
     <t>SR-KB-01</t>
   </si>
   <si>
-    <t>The system shall use a database to store approved Apple UI/UX course knowledge, assignment deadlines and approved RMIT information.</t>
-  </si>
-  <si>
     <t>Database solution discussed with and accepted by client.</t>
   </si>
   <si>
     <t>SR-KB-02</t>
   </si>
   <si>
-    <t>The system shall answer supported UI/UX concept questions using information available to the approved knowledge system.</t>
-  </si>
-  <si>
     <t>Core client use case.</t>
   </si>
   <si>
@@ -296,9 +272,6 @@
     <t>SR-KB-04</t>
   </si>
   <si>
-    <t>The approved RMIT information scope shall include course-related information, campus/location information, student services, academic policies, special consideration information and general RMIT FAQs.</t>
-  </si>
-  <si>
     <t>User confirmed all identified categories are required.</t>
   </si>
   <si>
@@ -314,9 +287,6 @@
     <t>SR-KB-06</t>
   </si>
   <si>
-    <t>Internet retrieval of RMIT information may be added using approved RMIT sources only.</t>
-  </si>
-  <si>
     <t>Proposed</t>
   </si>
   <si>
@@ -396,9 +366,6 @@
   </si>
   <si>
     <t>SR-RES-03</t>
-  </si>
-  <si>
-    <t>When the iPad fallback is being used, the returned answer shall be displayed as readable text on the iPad.</t>
   </si>
   <si>
     <t>Client-defined fallback behaviour.</t>
@@ -457,45 +424,24 @@
     <t>SR-ADM-01</t>
   </si>
   <si>
-    <t>An authenticated Admin shall be able to add approved course knowledge to the knowledge database.</t>
-  </si>
-  <si>
     <t>SR-ADM-02</t>
   </si>
   <si>
-    <t>An authenticated Admin shall be able to edit or remove course knowledge stored in the database.</t>
-  </si>
-  <si>
     <t>SR-ADM-03</t>
   </si>
   <si>
-    <t>An authenticated Admin shall be able to add or update assignment deadline information.</t>
-  </si>
-  <si>
     <t>Required to keep administrative answers current.</t>
   </si>
   <si>
     <t>SR-ADM-04</t>
   </si>
   <si>
-    <t>An authenticated Admin shall be able to add or update approved RMIT information.</t>
-  </si>
-  <si>
-    <t>Database-management requirement.</t>
-  </si>
-  <si>
     <t>SR-ADM-05</t>
   </si>
   <si>
     <t>An authenticated Admin shall be able to view recorded student enquiry records that the agreed data-retention policy permits the system to store.</t>
   </si>
   <si>
-    <t>Confirmed/TBC dependency</t>
-  </si>
-  <si>
-    <t>Function confirmed; exact stored data is not yet agreed.</t>
-  </si>
-  <si>
     <t>SR-ADM-06</t>
   </si>
   <si>
@@ -503,9 +449,6 @@
   </si>
   <si>
     <t>Supports knowledge-base improvement.</t>
-  </si>
-  <si>
-    <t>SR-ADM-07</t>
   </si>
   <si>
     <t>An authenticated Admin shall be able to create, disable and manage Admin/Developer user accounts.</t>
@@ -615,10 +558,6 @@
     <t>NFR-02</t>
   </si>
   <si>
-    <t>Core speech-to-text and LLM processing shall execute on the client's Mac Studio rather than requiring a cloud-hosted LLM service.</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
     <t>Confirmed</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
@@ -628,6 +567,78 @@
   </si>
   <si>
     <t>Derived</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>IPad shall convert a received audio recording into text before sending to the MCP server and call LLM.</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>The captured audio file should be converted to text in ipad before sending to MCP server.</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Each submitted audio text request shall receive a success or failure response from the backend.</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>NAO shall be the primary student voice-input device when the robot is technically operational.</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>NAO shall capture a student's spoken enquiry as an audio recording suitable for transmission to the ipad and then backend.</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>If NAO cannot be made operational, the system shall support an iPad fallback that can record student audio, tranfer the recording to text and send to MCP server running on the Mac Studio and display the returned text response.</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>The system shall use a database or obsidian to store course information, assignment deadlines. Should use web search to get RMIT inforamtion. Should train AI model to anwser UIUX related questions.</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>The approved RMIT information scope shall include course-related information, campus/location information, student services, academic policies, special consideration information and general RMIT FAQs.</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Internet retrieval of RMIT information must use approved RMIT sources only.</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>The system shall answer supported UI/UX concept questions using well trained AI model.</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>When the iPad fallback is being used, the returned answer shall be readed out by the iPad.</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>An authenticated Admin shall be able to add approved course information to the knowledge database(obsidian).</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>An authenticated Admin shall be able to edit or remove course information stored in the database/obsidian.</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>An authenticated Admin shall be able to add or update assignment deadline information.</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Could</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t xml:space="preserve">TBC </t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>TBC</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Core LLM processing shall execute on the client's Mac Studio rather than requiring a cloud-hosted LLM service.</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
 </sst>
@@ -726,20 +737,20 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1030,16 +1041,16 @@
     <col min="5" max="5" width="33.1640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" s="4" customFormat="1" ht="55" customHeight="1">
-      <c r="A1" s="5" t="s">
+    <row r="1" spans="1:5" s="3" customFormat="1" ht="55" customHeight="1">
+      <c r="A1" s="7" t="s">
         <v>29</v>
       </c>
-      <c r="B1" s="5"/>
-      <c r="C1" s="5"/>
-      <c r="D1" s="5"/>
-      <c r="E1" s="5"/>
-    </row>
-    <row r="2" spans="1:5" s="4" customFormat="1" ht="55" customHeight="1">
+      <c r="B1" s="7"/>
+      <c r="C1" s="7"/>
+      <c r="D1" s="7"/>
+      <c r="E1" s="7"/>
+    </row>
+    <row r="2" spans="1:5" s="3" customFormat="1" ht="55" customHeight="1">
       <c r="A2" s="1" t="s">
         <v>0</v>
       </c>
@@ -1056,7 +1067,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="3" spans="1:5" s="4" customFormat="1" ht="55" customHeight="1">
+    <row r="3" spans="1:5" s="3" customFormat="1" ht="55" customHeight="1">
       <c r="A3" s="2" t="s">
         <v>5</v>
       </c>
@@ -1073,7 +1084,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="4" spans="1:5" s="4" customFormat="1" ht="55" customHeight="1">
+    <row r="4" spans="1:5" s="3" customFormat="1" ht="55" customHeight="1">
       <c r="A4" s="2" t="s">
         <v>10</v>
       </c>
@@ -1090,7 +1101,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="5" spans="1:5" s="4" customFormat="1" ht="55" customHeight="1">
+    <row r="5" spans="1:5" s="3" customFormat="1" ht="55" customHeight="1">
       <c r="A5" s="2" t="s">
         <v>14</v>
       </c>
@@ -1107,7 +1118,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:5" s="4" customFormat="1" ht="55" customHeight="1">
+    <row r="6" spans="1:5" s="3" customFormat="1" ht="55" customHeight="1">
       <c r="A6" s="2" t="s">
         <v>17</v>
       </c>
@@ -1124,7 +1135,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="7" spans="1:5" s="4" customFormat="1" ht="55" customHeight="1">
+    <row r="7" spans="1:5" s="3" customFormat="1" ht="55" customHeight="1">
       <c r="A7" s="2" t="s">
         <v>20</v>
       </c>
@@ -1141,7 +1152,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="8" spans="1:5" s="4" customFormat="1" ht="55" customHeight="1">
+    <row r="8" spans="1:5" s="3" customFormat="1" ht="55" customHeight="1">
       <c r="A8" s="2" t="s">
         <v>23</v>
       </c>
@@ -1158,7 +1169,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="9" spans="1:5" s="4" customFormat="1" ht="55" customHeight="1">
+    <row r="9" spans="1:5" s="3" customFormat="1" ht="55" customHeight="1">
       <c r="A9" s="2" t="s">
         <v>26</v>
       </c>
@@ -1194,43 +1205,43 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
-      <c r="A1" s="3" t="s">
-        <v>164</v>
-      </c>
-      <c r="B1" s="3"/>
-      <c r="C1" s="3"/>
+      <c r="A1" s="6" t="s">
+        <v>145</v>
+      </c>
+      <c r="B1" s="6"/>
+      <c r="C1" s="6"/>
     </row>
     <row r="2" spans="1:3">
-      <c r="A2" s="6" t="s">
+      <c r="A2" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="6" t="s">
-        <v>51</v>
-      </c>
-      <c r="C2" s="6" t="s">
+      <c r="B2" s="4" t="s">
+        <v>46</v>
+      </c>
+      <c r="C2" s="4" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="3" spans="1:3" ht="42">
-      <c r="A3" s="7" t="s">
-        <v>165</v>
+      <c r="A3" s="5" t="s">
+        <v>146</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>167</v>
-      </c>
-      <c r="C3" s="7" t="s">
         <v>168</v>
       </c>
+      <c r="C3" s="5" t="s">
+        <v>148</v>
+      </c>
     </row>
     <row r="4" spans="1:3" ht="42">
-      <c r="A4" s="7" t="s">
-        <v>166</v>
+      <c r="A4" s="5" t="s">
+        <v>147</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>169</v>
-      </c>
-      <c r="C4" s="7" t="s">
-        <v>170</v>
+        <v>149</v>
+      </c>
+      <c r="C4" s="5" t="s">
+        <v>150</v>
       </c>
     </row>
   </sheetData>
@@ -1255,28 +1266,28 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="55" customHeight="1">
-      <c r="A1" s="5" t="s">
-        <v>49</v>
-      </c>
-      <c r="B1" s="5"/>
-      <c r="C1" s="5"/>
-      <c r="D1" s="5"/>
-      <c r="E1" s="5"/>
+      <c r="A1" s="7" t="s">
+        <v>44</v>
+      </c>
+      <c r="B1" s="7"/>
+      <c r="C1" s="7"/>
+      <c r="D1" s="7"/>
+      <c r="E1" s="7"/>
     </row>
     <row r="2" spans="1:5" ht="55" customHeight="1">
-      <c r="A2" s="6" t="s">
+      <c r="A2" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="6" t="s">
+      <c r="B2" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="6" t="s">
+      <c r="C2" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="D2" s="6" t="s">
+      <c r="D2" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="E2" s="6" t="s">
+      <c r="E2" s="4" t="s">
         <v>4</v>
       </c>
     </row>
@@ -1285,41 +1296,41 @@
         <v>30</v>
       </c>
       <c r="B3" s="2" t="s">
+        <v>154</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E3" s="2" t="s">
         <v>31</v>
-      </c>
-      <c r="C3" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="D3" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E3" s="2" t="s">
-        <v>32</v>
       </c>
     </row>
     <row r="4" spans="1:5" ht="55" customHeight="1">
       <c r="A4" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>155</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E4" s="2" t="s">
         <v>33</v>
-      </c>
-      <c r="B4" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="D4" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E4" s="2" t="s">
-        <v>35</v>
       </c>
     </row>
     <row r="5" spans="1:5" ht="55" customHeight="1">
       <c r="A5" s="2" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>37</v>
+        <v>152</v>
       </c>
       <c r="C5" s="2" t="s">
         <v>7</v>
@@ -1328,15 +1339,15 @@
         <v>8</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
     </row>
     <row r="6" spans="1:5" ht="55" customHeight="1">
       <c r="A6" s="2" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>40</v>
+        <v>153</v>
       </c>
       <c r="C6" s="2" t="s">
         <v>7</v>
@@ -1345,41 +1356,41 @@
         <v>12</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
     </row>
     <row r="7" spans="1:5" ht="55" customHeight="1">
       <c r="A7" s="2" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>43</v>
+        <v>156</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>50</v>
+        <v>45</v>
       </c>
       <c r="D7" s="2" t="s">
         <v>8</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>44</v>
+        <v>39</v>
       </c>
     </row>
     <row r="8" spans="1:5" ht="55" customHeight="1">
       <c r="A8" s="2" t="s">
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>46</v>
+        <v>41</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>47</v>
+        <v>42</v>
       </c>
       <c r="D8" s="2" t="s">
         <v>8</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>48</v>
+        <v>43</v>
       </c>
     </row>
   </sheetData>
@@ -1403,37 +1414,37 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="35" customHeight="1">
-      <c r="A1" s="5" t="s">
-        <v>61</v>
-      </c>
-      <c r="B1" s="5"/>
-      <c r="C1" s="5"/>
-      <c r="D1" s="5"/>
-      <c r="E1" s="5"/>
+      <c r="A1" s="7" t="s">
+        <v>55</v>
+      </c>
+      <c r="B1" s="7"/>
+      <c r="C1" s="7"/>
+      <c r="D1" s="7"/>
+      <c r="E1" s="7"/>
     </row>
     <row r="2" spans="1:5" ht="35" customHeight="1">
-      <c r="A2" s="6" t="s">
+      <c r="A2" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="6" t="s">
-        <v>51</v>
-      </c>
-      <c r="C2" s="6" t="s">
+      <c r="B2" s="4" t="s">
+        <v>46</v>
+      </c>
+      <c r="C2" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="D2" s="6" t="s">
+      <c r="D2" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="E2" s="6" t="s">
+      <c r="E2" s="4" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="3" spans="1:5" ht="35" customHeight="1">
       <c r="A3" s="2" t="s">
-        <v>52</v>
+        <v>47</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>53</v>
+        <v>151</v>
       </c>
       <c r="C3" s="2" t="s">
         <v>7</v>
@@ -1442,15 +1453,15 @@
         <v>8</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>54</v>
+        <v>48</v>
       </c>
     </row>
     <row r="4" spans="1:5" ht="35" customHeight="1">
       <c r="A4" s="2" t="s">
-        <v>55</v>
+        <v>49</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>56</v>
+        <v>50</v>
       </c>
       <c r="C4" s="2" t="s">
         <v>7</v>
@@ -1459,15 +1470,15 @@
         <v>12</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>57</v>
+        <v>51</v>
       </c>
     </row>
     <row r="5" spans="1:5" ht="35" customHeight="1">
       <c r="A5" s="2" t="s">
-        <v>58</v>
+        <v>52</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>59</v>
+        <v>53</v>
       </c>
       <c r="C5" s="2" t="s">
         <v>7</v>
@@ -1476,7 +1487,7 @@
         <v>12</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>60</v>
+        <v>54</v>
       </c>
     </row>
   </sheetData>
@@ -1500,37 +1511,37 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="55" customHeight="1">
-      <c r="A1" s="5" t="s">
-        <v>74</v>
-      </c>
-      <c r="B1" s="5"/>
-      <c r="C1" s="5"/>
-      <c r="D1" s="5"/>
-      <c r="E1" s="5"/>
+      <c r="A1" s="7" t="s">
+        <v>68</v>
+      </c>
+      <c r="B1" s="7"/>
+      <c r="C1" s="7"/>
+      <c r="D1" s="7"/>
+      <c r="E1" s="7"/>
     </row>
     <row r="2" spans="1:5" ht="55" customHeight="1">
-      <c r="A2" s="6" t="s">
+      <c r="A2" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="6" t="s">
-        <v>51</v>
-      </c>
-      <c r="C2" s="6" t="s">
+      <c r="B2" s="4" t="s">
+        <v>46</v>
+      </c>
+      <c r="C2" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="D2" s="6" t="s">
+      <c r="D2" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="E2" s="6" t="s">
+      <c r="E2" s="4" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="3" spans="1:5" ht="55" customHeight="1">
       <c r="A3" s="2" t="s">
-        <v>62</v>
+        <v>56</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>63</v>
+        <v>57</v>
       </c>
       <c r="C3" s="2" t="s">
         <v>7</v>
@@ -1539,15 +1550,15 @@
         <v>8</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>64</v>
+        <v>58</v>
       </c>
     </row>
     <row r="4" spans="1:5" ht="55" customHeight="1">
       <c r="A4" s="2" t="s">
-        <v>65</v>
+        <v>59</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>66</v>
+        <v>60</v>
       </c>
       <c r="C4" s="2" t="s">
         <v>7</v>
@@ -1556,15 +1567,15 @@
         <v>8</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>67</v>
+        <v>61</v>
       </c>
     </row>
     <row r="5" spans="1:5" ht="55" customHeight="1">
       <c r="A5" s="2" t="s">
-        <v>68</v>
+        <v>62</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>69</v>
+        <v>63</v>
       </c>
       <c r="C5" s="2" t="s">
         <v>7</v>
@@ -1573,15 +1584,15 @@
         <v>8</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>70</v>
+        <v>64</v>
       </c>
     </row>
     <row r="6" spans="1:5" ht="55" customHeight="1">
       <c r="A6" s="2" t="s">
-        <v>71</v>
+        <v>65</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>72</v>
+        <v>66</v>
       </c>
       <c r="C6" s="2" t="s">
         <v>7</v>
@@ -1590,7 +1601,7 @@
         <v>8</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
     </row>
   </sheetData>
@@ -1615,37 +1626,37 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="55" customHeight="1">
-      <c r="A1" s="5" t="s">
-        <v>95</v>
-      </c>
-      <c r="B1" s="5"/>
-      <c r="C1" s="5"/>
-      <c r="D1" s="5"/>
-      <c r="E1" s="5"/>
+      <c r="A1" s="7" t="s">
+        <v>85</v>
+      </c>
+      <c r="B1" s="7"/>
+      <c r="C1" s="7"/>
+      <c r="D1" s="7"/>
+      <c r="E1" s="7"/>
     </row>
     <row r="2" spans="1:5" ht="55" customHeight="1">
-      <c r="A2" s="6" t="s">
+      <c r="A2" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="6" t="s">
-        <v>51</v>
-      </c>
-      <c r="C2" s="6" t="s">
+      <c r="B2" s="4" t="s">
+        <v>46</v>
+      </c>
+      <c r="C2" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="D2" s="6" t="s">
+      <c r="D2" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="E2" s="6" t="s">
+      <c r="E2" s="4" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="3" spans="1:5" ht="55" customHeight="1">
       <c r="A3" s="2" t="s">
-        <v>75</v>
+        <v>69</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>76</v>
+        <v>157</v>
       </c>
       <c r="C3" s="2" t="s">
         <v>7</v>
@@ -1654,15 +1665,15 @@
         <v>8</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>77</v>
+        <v>70</v>
       </c>
     </row>
     <row r="4" spans="1:5" ht="55" customHeight="1">
       <c r="A4" s="2" t="s">
-        <v>78</v>
+        <v>71</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>79</v>
+        <v>160</v>
       </c>
       <c r="C4" s="2" t="s">
         <v>7</v>
@@ -1671,15 +1682,15 @@
         <v>8</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>80</v>
+        <v>72</v>
       </c>
     </row>
     <row r="5" spans="1:5" ht="55" customHeight="1">
       <c r="A5" s="2" t="s">
-        <v>81</v>
+        <v>73</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>82</v>
+        <v>74</v>
       </c>
       <c r="C5" s="2" t="s">
         <v>7</v>
@@ -1688,15 +1699,15 @@
         <v>12</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>83</v>
+        <v>75</v>
       </c>
     </row>
     <row r="6" spans="1:5" ht="55" customHeight="1">
       <c r="A6" s="2" t="s">
-        <v>84</v>
+        <v>76</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>85</v>
+        <v>158</v>
       </c>
       <c r="C6" s="2" t="s">
         <v>7</v>
@@ -1705,15 +1716,15 @@
         <v>8</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>86</v>
+        <v>77</v>
       </c>
     </row>
     <row r="7" spans="1:5" ht="55" customHeight="1">
       <c r="A7" s="2" t="s">
-        <v>87</v>
+        <v>78</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>88</v>
+        <v>79</v>
       </c>
       <c r="C7" s="2" t="s">
         <v>7</v>
@@ -1722,24 +1733,24 @@
         <v>12</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>89</v>
+        <v>80</v>
       </c>
     </row>
     <row r="8" spans="1:5" ht="55" customHeight="1">
       <c r="A8" s="2" t="s">
-        <v>90</v>
+        <v>81</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>91</v>
+        <v>159</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>92</v>
+        <v>82</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>93</v>
+        <v>83</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>94</v>
+        <v>84</v>
       </c>
     </row>
   </sheetData>
@@ -1763,37 +1774,37 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="55" customHeight="1">
-      <c r="A1" s="5" t="s">
-        <v>109</v>
-      </c>
-      <c r="B1" s="5"/>
-      <c r="C1" s="5"/>
-      <c r="D1" s="5"/>
-      <c r="E1" s="5"/>
+      <c r="A1" s="7" t="s">
+        <v>99</v>
+      </c>
+      <c r="B1" s="7"/>
+      <c r="C1" s="7"/>
+      <c r="D1" s="7"/>
+      <c r="E1" s="7"/>
     </row>
     <row r="2" spans="1:5" ht="55" customHeight="1">
-      <c r="A2" s="6" t="s">
+      <c r="A2" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="6" t="s">
-        <v>51</v>
-      </c>
-      <c r="C2" s="6" t="s">
+      <c r="B2" s="4" t="s">
+        <v>46</v>
+      </c>
+      <c r="C2" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="D2" s="6" t="s">
+      <c r="D2" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="E2" s="6" t="s">
+      <c r="E2" s="4" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="3" spans="1:5" ht="55" customHeight="1">
       <c r="A3" s="2" t="s">
-        <v>96</v>
+        <v>86</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>97</v>
+        <v>87</v>
       </c>
       <c r="C3" s="2" t="s">
         <v>7</v>
@@ -1802,15 +1813,15 @@
         <v>8</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>98</v>
+        <v>88</v>
       </c>
     </row>
     <row r="4" spans="1:5" ht="55" customHeight="1">
       <c r="A4" s="2" t="s">
-        <v>99</v>
+        <v>89</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>100</v>
+        <v>90</v>
       </c>
       <c r="C4" s="2" t="s">
         <v>7</v>
@@ -1819,15 +1830,15 @@
         <v>8</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>101</v>
+        <v>91</v>
       </c>
     </row>
     <row r="5" spans="1:5" ht="55" customHeight="1">
       <c r="A5" s="2" t="s">
-        <v>102</v>
+        <v>92</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>103</v>
+        <v>93</v>
       </c>
       <c r="C5" s="2" t="s">
         <v>7</v>
@@ -1836,15 +1847,15 @@
         <v>8</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>104</v>
+        <v>94</v>
       </c>
     </row>
     <row r="6" spans="1:5" ht="55" customHeight="1">
       <c r="A6" s="2" t="s">
-        <v>105</v>
+        <v>95</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>106</v>
+        <v>96</v>
       </c>
       <c r="C6" s="2" t="s">
         <v>7</v>
@@ -1853,24 +1864,24 @@
         <v>8</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>104</v>
+        <v>94</v>
       </c>
     </row>
     <row r="7" spans="1:5" ht="55" customHeight="1">
       <c r="A7" s="2" t="s">
-        <v>107</v>
+        <v>97</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>108</v>
+        <v>98</v>
       </c>
       <c r="C7" s="2" t="s">
         <v>7</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>93</v>
+        <v>83</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>110</v>
+        <v>100</v>
       </c>
     </row>
   </sheetData>
@@ -1895,37 +1906,37 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="55" customHeight="1">
-      <c r="A1" s="5" t="s">
-        <v>126</v>
-      </c>
-      <c r="B1" s="5"/>
-      <c r="C1" s="5"/>
-      <c r="D1" s="5"/>
-      <c r="E1" s="5"/>
+      <c r="A1" s="7" t="s">
+        <v>115</v>
+      </c>
+      <c r="B1" s="7"/>
+      <c r="C1" s="7"/>
+      <c r="D1" s="7"/>
+      <c r="E1" s="7"/>
     </row>
     <row r="2" spans="1:5" ht="55" customHeight="1">
-      <c r="A2" s="6" t="s">
+      <c r="A2" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="6" t="s">
-        <v>51</v>
-      </c>
-      <c r="C2" s="6" t="s">
+      <c r="B2" s="4" t="s">
+        <v>46</v>
+      </c>
+      <c r="C2" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="D2" s="6" t="s">
+      <c r="D2" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="E2" s="6" t="s">
+      <c r="E2" s="4" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="3" spans="1:5" ht="55" customHeight="1">
       <c r="A3" s="2" t="s">
-        <v>111</v>
+        <v>101</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>112</v>
+        <v>102</v>
       </c>
       <c r="C3" s="2" t="s">
         <v>7</v>
@@ -1934,15 +1945,15 @@
         <v>8</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>113</v>
+        <v>103</v>
       </c>
     </row>
     <row r="4" spans="1:5" ht="55" customHeight="1">
       <c r="A4" s="2" t="s">
-        <v>114</v>
+        <v>104</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>115</v>
+        <v>105</v>
       </c>
       <c r="C4" s="2" t="s">
         <v>7</v>
@@ -1951,32 +1962,32 @@
         <v>8</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>116</v>
+        <v>106</v>
       </c>
     </row>
     <row r="5" spans="1:5" ht="55" customHeight="1">
       <c r="A5" s="2" t="s">
-        <v>117</v>
+        <v>107</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>118</v>
+        <v>161</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>127</v>
+        <v>116</v>
       </c>
       <c r="D5" s="2" t="s">
         <v>8</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>119</v>
+        <v>108</v>
       </c>
     </row>
     <row r="6" spans="1:5" ht="55" customHeight="1">
       <c r="A6" s="2" t="s">
-        <v>120</v>
+        <v>109</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>121</v>
+        <v>110</v>
       </c>
       <c r="C6" s="2" t="s">
         <v>7</v>
@@ -1985,15 +1996,15 @@
         <v>8</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>122</v>
+        <v>111</v>
       </c>
     </row>
     <row r="7" spans="1:5" ht="55" customHeight="1">
       <c r="A7" s="2" t="s">
-        <v>123</v>
+        <v>112</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>124</v>
+        <v>113</v>
       </c>
       <c r="C7" s="2" t="s">
         <v>7</v>
@@ -2002,7 +2013,7 @@
         <v>12</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>125</v>
+        <v>114</v>
       </c>
     </row>
   </sheetData>
@@ -2026,37 +2037,37 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="35" customHeight="1">
-      <c r="A1" s="5" t="s">
-        <v>148</v>
-      </c>
-      <c r="B1" s="5"/>
-      <c r="C1" s="5"/>
-      <c r="D1" s="5"/>
-      <c r="E1" s="5"/>
+      <c r="A1" s="7" t="s">
+        <v>129</v>
+      </c>
+      <c r="B1" s="7"/>
+      <c r="C1" s="7"/>
+      <c r="D1" s="7"/>
+      <c r="E1" s="7"/>
     </row>
     <row r="2" spans="1:5" ht="35" customHeight="1">
-      <c r="A2" s="6" t="s">
+      <c r="A2" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="6" t="s">
-        <v>51</v>
-      </c>
-      <c r="C2" s="6" t="s">
+      <c r="B2" s="4" t="s">
+        <v>46</v>
+      </c>
+      <c r="C2" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="D2" s="6" t="s">
+      <c r="D2" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="E2" s="6" t="s">
+      <c r="E2" s="4" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="3" spans="1:5" ht="35" customHeight="1">
       <c r="A3" s="2" t="s">
-        <v>128</v>
+        <v>117</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>129</v>
+        <v>162</v>
       </c>
       <c r="C3" s="2" t="s">
         <v>7</v>
@@ -2065,15 +2076,15 @@
         <v>8</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>101</v>
+        <v>91</v>
       </c>
     </row>
     <row r="4" spans="1:5" ht="35" customHeight="1">
       <c r="A4" s="2" t="s">
-        <v>130</v>
+        <v>118</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>131</v>
+        <v>163</v>
       </c>
       <c r="C4" s="2" t="s">
         <v>7</v>
@@ -2082,15 +2093,15 @@
         <v>8</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>101</v>
+        <v>91</v>
       </c>
     </row>
     <row r="5" spans="1:5" ht="35" customHeight="1">
       <c r="A5" s="2" t="s">
-        <v>132</v>
+        <v>119</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>133</v>
+        <v>164</v>
       </c>
       <c r="C5" s="2" t="s">
         <v>7</v>
@@ -2099,49 +2110,49 @@
         <v>8</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>134</v>
+        <v>120</v>
       </c>
     </row>
     <row r="6" spans="1:5" ht="35" customHeight="1">
       <c r="A6" s="2" t="s">
-        <v>135</v>
+        <v>121</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>136</v>
+        <v>123</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>7</v>
+        <v>165</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>8</v>
+        <v>166</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>137</v>
+        <v>167</v>
       </c>
     </row>
     <row r="7" spans="1:5" ht="35" customHeight="1">
       <c r="A7" s="2" t="s">
-        <v>138</v>
+        <v>122</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>139</v>
+        <v>125</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>7</v>
+        <v>165</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>140</v>
+        <v>12</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>141</v>
+        <v>126</v>
       </c>
     </row>
     <row r="8" spans="1:5" ht="35" customHeight="1">
       <c r="A8" s="2" t="s">
-        <v>142</v>
+        <v>124</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>143</v>
+        <v>127</v>
       </c>
       <c r="C8" s="2" t="s">
         <v>7</v>
@@ -2150,26 +2161,10 @@
         <v>8</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5" ht="35" customHeight="1">
-      <c r="A9" s="2" t="s">
-        <v>145</v>
-      </c>
-      <c r="B9" s="2" t="s">
-        <v>146</v>
-      </c>
-      <c r="C9" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="D9" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E9" s="2" t="s">
-        <v>147</v>
-      </c>
-    </row>
+        <v>128</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" ht="35" customHeight="1"/>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:E1"/>
@@ -2191,37 +2186,37 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="35" customHeight="1">
-      <c r="A1" s="3" t="s">
-        <v>163</v>
-      </c>
-      <c r="B1" s="3"/>
-      <c r="C1" s="3"/>
-      <c r="D1" s="3"/>
-      <c r="E1" s="3"/>
+      <c r="A1" s="6" t="s">
+        <v>144</v>
+      </c>
+      <c r="B1" s="6"/>
+      <c r="C1" s="6"/>
+      <c r="D1" s="6"/>
+      <c r="E1" s="6"/>
     </row>
     <row r="2" spans="1:5" ht="35" customHeight="1">
-      <c r="A2" s="6" t="s">
+      <c r="A2" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="6" t="s">
-        <v>51</v>
-      </c>
-      <c r="C2" s="6" t="s">
+      <c r="B2" s="4" t="s">
+        <v>46</v>
+      </c>
+      <c r="C2" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="D2" s="6" t="s">
+      <c r="D2" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="E2" s="6" t="s">
+      <c r="E2" s="4" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="3" spans="1:5" ht="35" customHeight="1">
       <c r="A3" s="2" t="s">
-        <v>149</v>
+        <v>130</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>150</v>
+        <v>131</v>
       </c>
       <c r="C3" s="2" t="s">
         <v>7</v>
@@ -2230,15 +2225,15 @@
         <v>8</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>151</v>
+        <v>132</v>
       </c>
     </row>
     <row r="4" spans="1:5" ht="35" customHeight="1">
       <c r="A4" s="2" t="s">
-        <v>152</v>
+        <v>133</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>153</v>
+        <v>134</v>
       </c>
       <c r="C4" s="2" t="s">
         <v>7</v>
@@ -2247,15 +2242,15 @@
         <v>8</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>154</v>
+        <v>135</v>
       </c>
     </row>
     <row r="5" spans="1:5" ht="35" customHeight="1">
       <c r="A5" s="2" t="s">
-        <v>155</v>
+        <v>136</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>156</v>
+        <v>137</v>
       </c>
       <c r="C5" s="2" t="s">
         <v>7</v>
@@ -2264,15 +2259,15 @@
         <v>8</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>151</v>
+        <v>132</v>
       </c>
     </row>
     <row r="6" spans="1:5" ht="35" customHeight="1">
       <c r="A6" s="2" t="s">
-        <v>157</v>
+        <v>138</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>158</v>
+        <v>139</v>
       </c>
       <c r="C6" s="2" t="s">
         <v>7</v>
@@ -2281,15 +2276,15 @@
         <v>8</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>159</v>
+        <v>140</v>
       </c>
     </row>
     <row r="7" spans="1:5" ht="35" customHeight="1">
       <c r="A7" s="2" t="s">
-        <v>160</v>
+        <v>141</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>161</v>
+        <v>142</v>
       </c>
       <c r="C7" s="2" t="s">
         <v>7</v>
@@ -2298,7 +2293,7 @@
         <v>12</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>162</v>
+        <v>143</v>
       </c>
     </row>
   </sheetData>
@@ -2308,213 +2303,4 @@
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
-</file>
-
-<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="文档" ma:contentTypeID="0x01010096DE152E2C6A8C42B049878071E35BFA" ma:contentTypeVersion="10" ma:contentTypeDescription="新建文档。" ma:contentTypeScope="" ma:versionID="8b6d8f78d00b9fa0757aa0514a4cc277">
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="26c2b24a-a057-4aca-9b64-9bcaa58ad00d" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="1b75832d24a06c53705b30ce07eaa500" ns2:_="">
-    <xsd:import namespace="26c2b24a-a057-4aca-9b64-9bcaa58ad00d"/>
-    <xsd:element name="properties">
-      <xsd:complexType>
-        <xsd:sequence>
-          <xsd:element name="documentManagement">
-            <xsd:complexType>
-              <xsd:all>
-                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
-                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
-              </xsd:all>
-            </xsd:complexType>
-          </xsd:element>
-        </xsd:sequence>
-      </xsd:complexType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="26c2b24a-a057-4aca-9b64-9bcaa58ad00d" elementFormDefault="qualified">
-    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <xsd:element name="MediaServiceMetadata" ma:index="8" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceFastMetadata" ma:index="9" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceSearchProperties" ma:index="10" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceDateTaken" ma:index="11" nillable="true" ma:displayName="MediaServiceDateTaken" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="13" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="图像标记" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="c921d02d-b337-4ce5-bd1c-22d9132a6b17" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
-      <xsd:complexType>
-        <xsd:sequence>
-          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
-        </xsd:sequence>
-      </xsd:complexType>
-    </xsd:element>
-    <xsd:element name="MediaServiceOCR" ma:index="14" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note">
-          <xsd:maxLength value="255"/>
-        </xsd:restriction>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceGenerationTime" ma:index="15" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceEventHashCode" ma:index="16" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaLengthInSeconds" ma:index="17" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Unknown"/>
-      </xsd:simpleType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
-    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
-    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
-    <xsd:element name="coreProperties" type="CT_coreProperties"/>
-    <xsd:complexType name="CT_coreProperties">
-      <xsd:all>
-        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="内容类型"/>
-        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="标题"/>
-        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
-          <xsd:annotation>
-            <xsd:documentation>
-                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
-                    </xsd:documentation>
-          </xsd:annotation>
-        </xsd:element>
-        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-      </xsd:all>
-    </xsd:complexType>
-  </xsd:schema>
-  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
-    <xs:element name="Person">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:DisplayName" minOccurs="0"/>
-          <xs:element ref="pc:AccountId" minOccurs="0"/>
-          <xs:element ref="pc:AccountType" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="DisplayName" type="xs:string"/>
-    <xs:element name="AccountId" type="xs:string"/>
-    <xs:element name="AccountType" type="xs:string"/>
-    <xs:element name="BDCAssociatedEntity">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
-        </xs:sequence>
-        <xs:attribute ref="pc:EntityNamespace"/>
-        <xs:attribute ref="pc:EntityName"/>
-        <xs:attribute ref="pc:SystemInstanceName"/>
-        <xs:attribute ref="pc:AssociationName"/>
-      </xs:complexType>
-    </xs:element>
-    <xs:attribute name="EntityNamespace" type="xs:string"/>
-    <xs:attribute name="EntityName" type="xs:string"/>
-    <xs:attribute name="SystemInstanceName" type="xs:string"/>
-    <xs:attribute name="AssociationName" type="xs:string"/>
-    <xs:element name="BDCEntity">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
-          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
-          <xs:element ref="pc:EntityId1" minOccurs="0"/>
-          <xs:element ref="pc:EntityId2" minOccurs="0"/>
-          <xs:element ref="pc:EntityId3" minOccurs="0"/>
-          <xs:element ref="pc:EntityId4" minOccurs="0"/>
-          <xs:element ref="pc:EntityId5" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="EntityDisplayName" type="xs:string"/>
-    <xs:element name="EntityInstanceReference" type="xs:string"/>
-    <xs:element name="EntityId1" type="xs:string"/>
-    <xs:element name="EntityId2" type="xs:string"/>
-    <xs:element name="EntityId3" type="xs:string"/>
-    <xs:element name="EntityId4" type="xs:string"/>
-    <xs:element name="EntityId5" type="xs:string"/>
-    <xs:element name="Terms">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="TermInfo">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:TermName" minOccurs="0"/>
-          <xs:element ref="pc:TermId" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="TermName" type="xs:string"/>
-    <xs:element name="TermId" type="xs:string"/>
-  </xs:schema>
-</ct:contentTypeSchema>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="26c2b24a-a057-4aca-9b64-9bcaa58ad00d">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8793362D-1A5E-4FB8-A7F5-F7EA8589218E}"/>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E040E6A7-E5C4-4C54-8592-552077D18A5E}"/>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5E6AE47F-A882-42D8-93EA-CF02E2348D48}"/>
 </file>
</xml_diff>